<commit_message>
Fixed Lever Arm for TVC and retuned based on performance. Also changed actuator models to limit overshoot when saturated for realism.
</commit_message>
<xml_diff>
--- a/Parameters/constants.xlsx
+++ b/Parameters/constants.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdd953d6be32cedf/Documents/PSP Active Controls/M-EKF Dev Files/params/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdd953d6be32cedf/Documents/PSP Active Controls/ASTRA Model 2 Repo/Parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC434ED6-389E-474C-BF7B-E80EDB48C4FC}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{524061AB-F6BF-4BC6-8873-9FB8D209C3BF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2580" yWindow="2580" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -427,7 +427,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>0.995</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -460,7 +460,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>0.6</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Tuning for initial ASTRAv2 flight tests, Addition of redux script v1
</commit_message>
<xml_diff>
--- a/Parameters/constants.xlsx
+++ b/Parameters/constants.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdd953d6be32cedf/Documents/PSP Active Controls/ASTRA Model 2 Repo/Parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{524061AB-F6BF-4BC6-8873-9FB8D209C3BF}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{87EAED42-475D-4B6D-825F-7491F9F8CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9136DF62-4182-441F-84FB-10EDEFFFBFBA}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="2580" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -427,7 +427,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>1.2490000000000001</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -438,7 +438,7 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>0.753</v>
+        <v>0.5</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -449,7 +449,7 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>9.81</v>
+        <v>9.8014500000000009</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -460,7 +460,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>